<commit_message>
Snapshot trade tracker state before restructure
</commit_message>
<xml_diff>
--- a/trade_tracker.xlsx
+++ b/trade_tracker.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S108"/>
+  <dimension ref="A1:S118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7025,6 +7025,706 @@
       <c r="S108" t="inlineStr">
         <is>
           <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="9" t="n">
+        <v>46043</v>
+      </c>
+      <c r="C109" s="9" t="n">
+        <v>46086.53839304398</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>TNA</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>93</v>
+      </c>
+      <c r="G109" t="n">
+        <v>54.745</v>
+      </c>
+      <c r="H109" t="n">
+        <v>52.82</v>
+      </c>
+      <c r="I109" t="n">
+        <v>5091.285</v>
+      </c>
+      <c r="J109" t="n">
+        <v>4912.26</v>
+      </c>
+      <c r="K109">
+        <f>J109-I109</f>
+        <v/>
+      </c>
+      <c r="L109" t="n">
+        <v>2</v>
+      </c>
+      <c r="M109">
+        <f>K109-L109</f>
+        <v/>
+      </c>
+      <c r="N109">
+        <f>M109/I109</f>
+        <v/>
+      </c>
+      <c r="O109" t="n">
+        <v>43</v>
+      </c>
+      <c r="P109">
+        <f>IF(M109&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="9" t="n">
+        <v>46064</v>
+      </c>
+      <c r="C110" s="9" t="n">
+        <v>46087.56565171296</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>FAS</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>35</v>
+      </c>
+      <c r="G110" t="n">
+        <v>154.19</v>
+      </c>
+      <c r="H110" t="n">
+        <v>133</v>
+      </c>
+      <c r="I110" t="n">
+        <v>5396.65</v>
+      </c>
+      <c r="J110" t="n">
+        <v>4655</v>
+      </c>
+      <c r="K110">
+        <f>J110-I110</f>
+        <v/>
+      </c>
+      <c r="L110" t="n">
+        <v>2</v>
+      </c>
+      <c r="M110">
+        <f>K110-L110</f>
+        <v/>
+      </c>
+      <c r="N110">
+        <f>M110/I110</f>
+        <v/>
+      </c>
+      <c r="O110" t="n">
+        <v>23</v>
+      </c>
+      <c r="P110">
+        <f>IF(M110&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="9" t="n">
+        <v>46044</v>
+      </c>
+      <c r="C111" s="9" t="n">
+        <v>46098.56915672454</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>11</v>
+      </c>
+      <c r="G111" t="n">
+        <v>443.6</v>
+      </c>
+      <c r="H111" t="n">
+        <v>460.43</v>
+      </c>
+      <c r="I111" t="n">
+        <v>4879.6</v>
+      </c>
+      <c r="J111" t="n">
+        <v>5064.73</v>
+      </c>
+      <c r="K111">
+        <f>J111-I111</f>
+        <v/>
+      </c>
+      <c r="L111" t="n">
+        <v>2</v>
+      </c>
+      <c r="M111">
+        <f>K111-L111</f>
+        <v/>
+      </c>
+      <c r="N111">
+        <f>M111/I111</f>
+        <v/>
+      </c>
+      <c r="O111" t="n">
+        <v>54</v>
+      </c>
+      <c r="P111">
+        <f>IF(M111&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="9" t="n">
+        <v>46097</v>
+      </c>
+      <c r="C112" s="9" t="n">
+        <v>46098.56915744213</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>LABU</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>35</v>
+      </c>
+      <c r="G112" t="n">
+        <v>148.85</v>
+      </c>
+      <c r="H112" t="n">
+        <v>156.24</v>
+      </c>
+      <c r="I112" t="n">
+        <v>5209.75</v>
+      </c>
+      <c r="J112" t="n">
+        <v>5468.400000000001</v>
+      </c>
+      <c r="K112">
+        <f>J112-I112</f>
+        <v/>
+      </c>
+      <c r="L112" t="n">
+        <v>2</v>
+      </c>
+      <c r="M112">
+        <f>K112-L112</f>
+        <v/>
+      </c>
+      <c r="N112">
+        <f>M112/I112</f>
+        <v/>
+      </c>
+      <c r="O112" t="n">
+        <v>1</v>
+      </c>
+      <c r="P112">
+        <f>IF(M112&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="9" t="n">
+        <v>46036</v>
+      </c>
+      <c r="C113" s="9" t="n">
+        <v>46098.88731337963</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>23</v>
+      </c>
+      <c r="G113" t="n">
+        <v>220.97</v>
+      </c>
+      <c r="H113" t="n">
+        <v>196.15</v>
+      </c>
+      <c r="I113" t="n">
+        <v>5082.31</v>
+      </c>
+      <c r="J113" t="n">
+        <v>4511.45</v>
+      </c>
+      <c r="K113">
+        <f>J113-I113</f>
+        <v/>
+      </c>
+      <c r="L113" t="n">
+        <v>2</v>
+      </c>
+      <c r="M113">
+        <f>K113-L113</f>
+        <v/>
+      </c>
+      <c r="N113">
+        <f>M113/I113</f>
+        <v/>
+      </c>
+      <c r="O113" t="n">
+        <v>62</v>
+      </c>
+      <c r="P113">
+        <f>IF(M113&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="9" t="n">
+        <v>46028</v>
+      </c>
+      <c r="C114" s="9" t="n">
+        <v>46100.47062840278</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>ERX</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>82</v>
+      </c>
+      <c r="G114" t="n">
+        <v>61.35</v>
+      </c>
+      <c r="H114" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="I114" t="n">
+        <v>5030.7</v>
+      </c>
+      <c r="J114" t="n">
+        <v>7667</v>
+      </c>
+      <c r="K114">
+        <f>J114-I114</f>
+        <v/>
+      </c>
+      <c r="L114" t="n">
+        <v>2</v>
+      </c>
+      <c r="M114">
+        <f>K114-L114</f>
+        <v/>
+      </c>
+      <c r="N114">
+        <f>M114/I114</f>
+        <v/>
+      </c>
+      <c r="O114" t="n">
+        <v>72</v>
+      </c>
+      <c r="P114">
+        <f>IF(M114&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="9" t="n">
+        <v>46042</v>
+      </c>
+      <c r="C115" s="9" t="n">
+        <v>46100.47062850695</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>20</v>
+      </c>
+      <c r="G115" t="n">
+        <v>243.95</v>
+      </c>
+      <c r="H115" t="n">
+        <v>249.94</v>
+      </c>
+      <c r="I115" t="n">
+        <v>4879</v>
+      </c>
+      <c r="J115" t="n">
+        <v>4998.8</v>
+      </c>
+      <c r="K115">
+        <f>J115-I115</f>
+        <v/>
+      </c>
+      <c r="L115" t="n">
+        <v>2</v>
+      </c>
+      <c r="M115">
+        <f>K115-L115</f>
+        <v/>
+      </c>
+      <c r="N115">
+        <f>M115/I115</f>
+        <v/>
+      </c>
+      <c r="O115" t="n">
+        <v>58</v>
+      </c>
+      <c r="P115">
+        <f>IF(M115&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="9" t="n">
+        <v>46044</v>
+      </c>
+      <c r="C116" s="9" t="n">
+        <v>46100.47062856481</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>8</v>
+      </c>
+      <c r="G116" t="n">
+        <v>647.63</v>
+      </c>
+      <c r="H116" t="n">
+        <v>615.6799999999999</v>
+      </c>
+      <c r="I116" t="n">
+        <v>5181.04</v>
+      </c>
+      <c r="J116" t="n">
+        <v>4925.44</v>
+      </c>
+      <c r="K116">
+        <f>J116-I116</f>
+        <v/>
+      </c>
+      <c r="L116" t="n">
+        <v>2</v>
+      </c>
+      <c r="M116">
+        <f>K116-L116</f>
+        <v/>
+      </c>
+      <c r="N116">
+        <f>M116/I116</f>
+        <v/>
+      </c>
+      <c r="O116" t="n">
+        <v>56</v>
+      </c>
+      <c r="P116">
+        <f>IF(M116&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="9" t="n">
+        <v>46097</v>
+      </c>
+      <c r="C117" s="9" t="n">
+        <v>46107.50928837963</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>UGL</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>72</v>
+      </c>
+      <c r="G117" t="n">
+        <v>71.48</v>
+      </c>
+      <c r="H117" t="n">
+        <v>57.71</v>
+      </c>
+      <c r="I117" t="n">
+        <v>5146.56</v>
+      </c>
+      <c r="J117" t="n">
+        <v>4155.12</v>
+      </c>
+      <c r="K117">
+        <f>J117-I117</f>
+        <v/>
+      </c>
+      <c r="L117" t="n">
+        <v>2</v>
+      </c>
+      <c r="M117">
+        <f>K117-L117</f>
+        <v/>
+      </c>
+      <c r="N117">
+        <f>M117/I117</f>
+        <v/>
+      </c>
+      <c r="O117" t="n">
+        <v>10</v>
+      </c>
+      <c r="P117">
+        <f>IF(M117&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="9" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C118" s="9" t="n">
+        <v>46134.64725333334</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>65</v>
+      </c>
+      <c r="G118" t="n">
+        <v>82.20999999999999</v>
+      </c>
+      <c r="H118" t="n">
+        <v>92.58</v>
+      </c>
+      <c r="I118" t="n">
+        <v>5343.65</v>
+      </c>
+      <c r="J118" t="n">
+        <v>6017.7</v>
+      </c>
+      <c r="K118">
+        <f>J118-I118</f>
+        <v/>
+      </c>
+      <c r="L118" t="n">
+        <v>2</v>
+      </c>
+      <c r="M118">
+        <f>K118-L118</f>
+        <v/>
+      </c>
+      <c r="N118">
+        <f>M118/I118</f>
+        <v/>
+      </c>
+      <c r="O118" t="n">
+        <v>71</v>
+      </c>
+      <c r="P118">
+        <f>IF(M118&gt;0,"Win","Loss")</f>
+        <v/>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>VPVMA</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>Universe Drop</t>
         </is>
       </c>
     </row>
@@ -7236,19 +7936,19 @@
         <v>46013</v>
       </c>
       <c r="E3" t="n">
-        <v>387.25</v>
+        <v>385.95</v>
       </c>
       <c r="F3" t="n">
         <v>4909.259999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>6583.25</v>
+        <v>6561.15</v>
       </c>
       <c r="H3" t="n">
-        <v>1673.990000000001</v>
+        <v>1651.89</v>
       </c>
       <c r="I3" t="n">
-        <v>0.340986217882125</v>
+        <v>0.3364845210887182</v>
       </c>
     </row>
     <row r="4">
@@ -7267,19 +7967,19 @@
         <v>46013</v>
       </c>
       <c r="E4" t="n">
-        <v>167</v>
+        <v>191.05</v>
       </c>
       <c r="F4" t="n">
         <v>4955.44</v>
       </c>
       <c r="G4" t="n">
-        <v>4676</v>
+        <v>5349.400000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>-279.4399999999996</v>
+        <v>393.9600000000009</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.05639055260481407</v>
+        <v>0.07950050853203772</v>
       </c>
     </row>
     <row r="5">
@@ -7298,19 +7998,19 @@
         <v>46014</v>
       </c>
       <c r="E5" t="n">
-        <v>45.5</v>
+        <v>65.27</v>
       </c>
       <c r="F5" t="n">
         <v>5019.059999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>6279</v>
+        <v>9007.26</v>
       </c>
       <c r="H5" t="n">
-        <v>1259.940000000001</v>
+        <v>3988.200000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2510310695628266</v>
+        <v>0.7946109430849602</v>
       </c>
     </row>
     <row r="6">
@@ -7329,19 +8029,19 @@
         <v>46027</v>
       </c>
       <c r="E6" t="n">
-        <v>676.7</v>
+        <v>555.4299999999999</v>
       </c>
       <c r="F6" t="n">
         <v>4970.7</v>
       </c>
       <c r="G6" t="n">
-        <v>6767</v>
+        <v>5554.299999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>1796.3</v>
+        <v>583.5999999999995</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3613776731647456</v>
+        <v>0.1174080109441324</v>
       </c>
     </row>
     <row r="7">
@@ -7360,454 +8060,426 @@
         <v>46027</v>
       </c>
       <c r="E7" t="n">
-        <v>861.7</v>
+        <v>934.84</v>
       </c>
       <c r="F7" t="n">
         <v>4571.7</v>
       </c>
       <c r="G7" t="n">
-        <v>4308.5</v>
+        <v>4674.2</v>
       </c>
       <c r="H7" t="n">
-        <v>-263.1999999999998</v>
+        <v>102.5</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.05757158168733733</v>
+        <v>0.02242054378021296</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ERX</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="C8" t="n">
-        <v>61.35</v>
+        <v>69.37</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46028</v>
+        <v>46030</v>
       </c>
       <c r="E8" t="n">
-        <v>89.34</v>
+        <v>74.63</v>
       </c>
       <c r="F8" t="n">
-        <v>5030.7</v>
+        <v>5064.01</v>
       </c>
       <c r="G8" t="n">
-        <v>7325.88</v>
+        <v>5447.99</v>
       </c>
       <c r="H8" t="n">
-        <v>2295.18</v>
+        <v>383.9799999999996</v>
       </c>
       <c r="I8" t="n">
-        <v>0.456234718826406</v>
+        <v>0.07582528470520389</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>73</v>
+        <v>199</v>
       </c>
       <c r="C9" t="n">
-        <v>69.37</v>
+        <v>26.5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46030</v>
+        <v>46049</v>
       </c>
       <c r="E9" t="n">
-        <v>80.22</v>
+        <v>26.8</v>
       </c>
       <c r="F9" t="n">
-        <v>5064.01</v>
+        <v>5273.5</v>
       </c>
       <c r="G9" t="n">
-        <v>5856.059999999999</v>
+        <v>5333.2</v>
       </c>
       <c r="H9" t="n">
-        <v>792.0499999999993</v>
+        <v>59.69999999999982</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1564076690211906</v>
+        <v>0.01132075471698113</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="C10" t="n">
-        <v>220.97</v>
+        <v>129.62</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46036</v>
+        <v>46051</v>
       </c>
       <c r="E10" t="n">
-        <v>198.62</v>
+        <v>103.07</v>
       </c>
       <c r="F10" t="n">
-        <v>5082.31</v>
+        <v>5314.42</v>
       </c>
       <c r="G10" t="n">
-        <v>4568.26</v>
+        <v>4225.87</v>
       </c>
       <c r="H10" t="n">
-        <v>-514.0500000000002</v>
+        <v>-1088.55</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.1011449518034122</v>
+        <v>-0.2048295016201205</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C11" t="n">
-        <v>243.95</v>
+        <v>153.63</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46042</v>
+        <v>46055</v>
       </c>
       <c r="E11" t="n">
-        <v>264.72</v>
+        <v>153.79</v>
       </c>
       <c r="F11" t="n">
-        <v>4879</v>
+        <v>5223.42</v>
       </c>
       <c r="G11" t="n">
-        <v>5294.400000000001</v>
+        <v>5228.86</v>
       </c>
       <c r="H11" t="n">
-        <v>415.4000000000005</v>
+        <v>5.4399999999996</v>
       </c>
       <c r="I11" t="n">
-        <v>0.08514039762246384</v>
+        <v>0.001041463255874397</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="C12" t="n">
-        <v>54.745</v>
+        <v>122.15</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46043</v>
+        <v>46063</v>
       </c>
       <c r="E12" t="n">
-        <v>54.23</v>
+        <v>129.73</v>
       </c>
       <c r="F12" t="n">
-        <v>5091.285</v>
+        <v>5374.6</v>
       </c>
       <c r="G12" t="n">
-        <v>5043.389999999999</v>
+        <v>5708.12</v>
       </c>
       <c r="H12" t="n">
-        <v>-47.89500000000044</v>
+        <v>333.5199999999995</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.00940725180381774</v>
+        <v>0.06205485059353233</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>TMF</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11</v>
+        <v>132</v>
       </c>
       <c r="C13" t="n">
-        <v>443.6</v>
+        <v>40.01</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46044</v>
+        <v>46076</v>
       </c>
       <c r="E13" t="n">
-        <v>490</v>
+        <v>36.28</v>
       </c>
       <c r="F13" t="n">
-        <v>4879.6</v>
+        <v>5281.32</v>
       </c>
       <c r="G13" t="n">
-        <v>5390</v>
+        <v>4788.96</v>
       </c>
       <c r="H13" t="n">
-        <v>510.3999999999996</v>
+        <v>-492.3599999999997</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1045987376014428</v>
+        <v>-0.09322669332666822</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C14" t="n">
-        <v>647.63</v>
+        <v>307.9</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>46044</v>
+        <v>46098</v>
       </c>
       <c r="E14" t="n">
-        <v>653.5599999999999</v>
+        <v>339.32</v>
       </c>
       <c r="F14" t="n">
-        <v>5181.04</v>
+        <v>5234.299999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>5228.48</v>
+        <v>5768.44</v>
       </c>
       <c r="H14" t="n">
-        <v>47.4399999999996</v>
+        <v>534.1400000000003</v>
       </c>
       <c r="I14" t="n">
-        <v>0.009156462795114395</v>
+        <v>0.102046118869763</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>199</v>
+        <v>16</v>
       </c>
       <c r="C15" t="n">
-        <v>26.5</v>
+        <v>320.995</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>46049</v>
+        <v>46098</v>
       </c>
       <c r="E15" t="n">
-        <v>27.26</v>
+        <v>422.65</v>
       </c>
       <c r="F15" t="n">
-        <v>5273.5</v>
+        <v>5135.92</v>
       </c>
       <c r="G15" t="n">
-        <v>5424.740000000001</v>
+        <v>6762.4</v>
       </c>
       <c r="H15" t="n">
-        <v>151.2400000000007</v>
+        <v>1626.48</v>
       </c>
       <c r="I15" t="n">
-        <v>0.02867924528301891</v>
+        <v>0.3166871758127072</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C16" t="n">
-        <v>129.62</v>
+        <v>208.34</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>46051</v>
+        <v>46100</v>
       </c>
       <c r="E16" t="n">
-        <v>109.42</v>
+        <v>200.5</v>
       </c>
       <c r="F16" t="n">
-        <v>5314.42</v>
+        <v>5208.5</v>
       </c>
       <c r="G16" t="n">
-        <v>4486.22</v>
+        <v>5012.5</v>
       </c>
       <c r="H16" t="n">
-        <v>-828.1999999999998</v>
+        <v>-196</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.1558401481252893</v>
+        <v>-0.03763079581453399</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>153.63</v>
+        <v>315.73</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>46055</v>
+        <v>46100</v>
       </c>
       <c r="E17" t="n">
-        <v>167.28</v>
+        <v>300.07</v>
       </c>
       <c r="F17" t="n">
-        <v>5223.42</v>
+        <v>5051.68</v>
       </c>
       <c r="G17" t="n">
-        <v>5687.52</v>
+        <v>4801.12</v>
       </c>
       <c r="H17" t="n">
-        <v>464.1000000000004</v>
+        <v>-250.5600000000004</v>
       </c>
       <c r="I17" t="n">
-        <v>0.08884983401679358</v>
+        <v>-0.04959934120926112</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>122.15</v>
+        <v>299.02</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>46063</v>
+        <v>46100</v>
       </c>
       <c r="E18" t="n">
-        <v>111.45</v>
+        <v>311.29</v>
       </c>
       <c r="F18" t="n">
-        <v>5374.6</v>
+        <v>5083.34</v>
       </c>
       <c r="G18" t="n">
-        <v>4903.8</v>
+        <v>5291.93</v>
       </c>
       <c r="H18" t="n">
-        <v>-470.8000000000002</v>
+        <v>208.5900000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.08759721653704468</v>
+        <v>0.04103404454551551</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="C19" t="n">
-        <v>82.20999999999999</v>
+        <v>246</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>46063</v>
+        <v>46100</v>
       </c>
       <c r="E19" t="n">
-        <v>97.09</v>
+        <v>255.94</v>
       </c>
       <c r="F19" t="n">
-        <v>5343.65</v>
+        <v>5166</v>
       </c>
       <c r="G19" t="n">
-        <v>6310.85</v>
+        <v>5374.74</v>
       </c>
       <c r="H19" t="n">
-        <v>967.2000000000007</v>
+        <v>208.7399999999998</v>
       </c>
       <c r="I19" t="n">
-        <v>0.1809998783602968</v>
+        <v>0.04040650406504054</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FAS</t>
+          <t>LABU</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C20" t="n">
-        <v>154.19</v>
+        <v>154.9</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>46064</v>
+        <v>46107</v>
       </c>
       <c r="E20" t="n">
-        <v>133.58</v>
+        <v>204.13</v>
       </c>
       <c r="F20" t="n">
-        <v>5396.65</v>
+        <v>4956.8</v>
       </c>
       <c r="G20" t="n">
-        <v>4675.3</v>
+        <v>6532.16</v>
       </c>
       <c r="H20" t="n">
-        <v>-721.3499999999995</v>
+        <v>1575.36</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.1336662559180232</v>
+        <v>0.317817947062621</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TMF</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>132</v>
-      </c>
-      <c r="C21" t="n">
-        <v>40.01</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>46076</v>
-      </c>
-      <c r="E21" t="n">
-        <v>40.53</v>
-      </c>
-      <c r="F21" t="n">
-        <v>5281.32</v>
-      </c>
-      <c r="G21" t="n">
-        <v>5349.96</v>
-      </c>
-      <c r="H21" t="n">
-        <v>68.64000000000033</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.01299675081229701</v>
-      </c>
+      <c r="D21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="D22" s="2" t="n"/>

</xml_diff>